<commit_message>
UPDATE codigo y README
</commit_message>
<xml_diff>
--- a/Inputs/Estaciones.xlsx
+++ b/Inputs/Estaciones.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\Datos_DGA\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE9A642-0160-4774-B1D7-E9C7EA2B0168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D71DFBF5-6FAB-4F6D-A383-E018ED5073A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2820" yWindow="720" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Estaciones DGA" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Estaciones</t>
   </si>
@@ -61,13 +72,31 @@
   </si>
   <si>
     <t>LOS LOROS</t>
+  </si>
+  <si>
+    <t>RIO ASTABURUAGA EN CONO</t>
+  </si>
+  <si>
+    <t>RIO BARROS NEGROS ANTES JUNTA VALLE ANCHO</t>
+  </si>
+  <si>
+    <t>RIO LAMAS EN EL SALTO</t>
+  </si>
+  <si>
+    <t>RIO VALLE ANCHO EN LA BARRERA</t>
+  </si>
+  <si>
+    <t>RIO VILLALOBOS EN VERTEDERO</t>
+  </si>
+  <si>
+    <t>RIO VALLE ANCHO ANTES  JUNTA BARROS NEGROS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,6 +112,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2328"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,9 +140,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,10 +424,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -454,6 +491,36 @@
         <v>11</v>
       </c>
     </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>